<commit_message>
using countif_ifs, sumif_ifs and many more
</commit_message>
<xml_diff>
--- a/Task.xlsx
+++ b/Task.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/657ac1910ce59299/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DSDA\Advanced Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D8195F1-A953-427A-9CB7-904A959F7CF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57FA3C2-73AB-4B8B-8FFC-6D7205742B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{C4E566D6-4848-4FA5-93A7-807593E85530}"/>
   </bookViews>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
   <si>
     <t>Name</t>
   </si>
@@ -72,6 +94,87 @@
   </si>
   <si>
     <t>Give 10% discount if both above conditions are met</t>
+  </si>
+  <si>
+    <t>Total Amount Based only on years</t>
+  </si>
+  <si>
+    <t>Marks</t>
+  </si>
+  <si>
+    <t>Ajit</t>
+  </si>
+  <si>
+    <t>Meena</t>
+  </si>
+  <si>
+    <t>Seema</t>
+  </si>
+  <si>
+    <t>Mayur</t>
+  </si>
+  <si>
+    <t>Ram</t>
+  </si>
+  <si>
+    <t>Umesh</t>
+  </si>
+  <si>
+    <t>Tina</t>
+  </si>
+  <si>
+    <t>Grades</t>
+  </si>
+  <si>
+    <t>&gt;=90</t>
+  </si>
+  <si>
+    <t>&gt;50</t>
+  </si>
+  <si>
+    <t>Average</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>&gt;40</t>
+  </si>
+  <si>
+    <t>Else</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Very Good</t>
+  </si>
+  <si>
+    <t>Rohan</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>&gt;=75</t>
+  </si>
+  <si>
+    <t>FORMULAS</t>
+  </si>
+  <si>
+    <t>ISTEXT</t>
+  </si>
+  <si>
+    <t>ISNUMBER</t>
+  </si>
+  <si>
+    <t>NOT FUNCTION</t>
+  </si>
+  <si>
+    <t>ISNA</t>
   </si>
 </sst>
 </file>
@@ -130,16 +233,94 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -469,13 +650,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F32760D1-5E6D-4E97-A7F4-910B353D760C}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="26.42578125" customWidth="1"/>
+    <col min="7" max="7" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -488,10 +675,14 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -502,10 +693,17 @@
         <v>2</v>
       </c>
       <c r="D2" s="3">
+        <f>IF(AND(B2&gt;=3000,C2&gt;=3),B2-(B2*0.1),B2)</f>
         <v>3500</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2">
+        <f>IF(C2&gt;3,0.9*B2,B2)</f>
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -516,10 +714,17 @@
         <v>4</v>
       </c>
       <c r="D3" s="3">
+        <f t="shared" ref="D3:D7" si="0">IF(AND(B3&gt;=3000,C3&gt;=3),B3-(B3*0.1),B3)</f>
         <v>2400</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3">
+        <f t="shared" ref="G3:G7" si="1">IF(C3&gt;3,0.9*B3,B3)</f>
+        <v>2160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
@@ -530,10 +735,17 @@
         <v>5</v>
       </c>
       <c r="D4" s="3">
+        <f t="shared" si="0"/>
         <v>4230</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4">
+        <f t="shared" si="1"/>
+        <v>4230</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
@@ -544,10 +756,17 @@
         <v>4</v>
       </c>
       <c r="D5" s="3">
+        <f t="shared" si="0"/>
         <v>5220</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>5220</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -558,10 +777,17 @@
         <v>6</v>
       </c>
       <c r="D6" s="3">
+        <f t="shared" si="0"/>
         <v>1500</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6">
+        <f t="shared" si="1"/>
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -572,10 +798,17 @@
         <v>3</v>
       </c>
       <c r="D7" s="3">
+        <f t="shared" si="0"/>
         <v>3150</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -585,8 +818,10 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -596,6 +831,274 @@
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="3">
+        <v>91</v>
+      </c>
+      <c r="C13" s="3" t="str">
+        <f>IF(ISTEXT(B13),"No Grade",IF(B13&gt;=90,"Excellent",IF(B13&gt;=75,"Very Good",IF(B13&gt;50,"Good",IF(B13&gt;40,"Average","Fail")))))</f>
+        <v>Excellent</v>
+      </c>
+      <c r="D13" s="3" t="str">
+        <f>IF(NOT(ISNUMBER(B13)),"No Data",IF(B13&gt;=90,"Excellent",IF(B13&gt;=75,"Very Good",IF(B13&gt;50,"Good",IF(B13&gt;40,"Average","Fail")))))</f>
+        <v>Excellent</v>
+      </c>
+      <c r="E13" s="3" t="str" cm="1">
+        <f t="array" ref="E13">_xlfn.IFS(ISTEXT(B13),"No  Data",B13&gt;=90,"Excellent",B13&gt;=75,"Very Good",B13&gt;50,"Good",B13&gt;40,"Average",B13&lt;40,"Fail")</f>
+        <v>Excellent</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="3">
+        <v>45</v>
+      </c>
+      <c r="C14" s="3" t="str">
+        <f t="shared" ref="C14:C22" si="2">IF(ISTEXT(B14),"No Grade",IF(B14&gt;=90,"Excellent",IF(B14&gt;=75,"Very Good",IF(B14&gt;50,"Good",IF(B14&gt;40,"Average","Fail")))))</f>
+        <v>Average</v>
+      </c>
+      <c r="D14" s="3" t="str">
+        <f t="shared" ref="D14:D22" si="3">IF(NOT(ISNUMBER(B14)),"No Data",IF(B14&gt;=90,"Excellent",IF(B14&gt;=75,"Very Good",IF(B14&gt;50,"Good",IF(B14&gt;40,"Average","Fail")))))</f>
+        <v>Average</v>
+      </c>
+      <c r="E14" s="3" t="str" cm="1">
+        <f t="array" ref="E14">_xlfn.IFS(ISTEXT(B14),"No  Data",B14&gt;=90,"Excellent",B14&gt;=75,"Very Good",B14&gt;50,"Good",B14&gt;40,"Average",B14&lt;40,"Fail")</f>
+        <v>Average</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" s="3">
+        <v>76</v>
+      </c>
+      <c r="C15" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Very Good</v>
+      </c>
+      <c r="D15" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>Very Good</v>
+      </c>
+      <c r="E15" s="3" t="str" cm="1">
+        <f t="array" ref="E15">_xlfn.IFS(ISTEXT(B15),"No  Data",B15&gt;=90,"Excellent",B15&gt;=75,"Very Good",B15&gt;50,"Good",B15&gt;40,"Average",B15&lt;40,"Fail")</f>
+        <v>Very Good</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="3">
+        <v>32</v>
+      </c>
+      <c r="C16" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Fail</v>
+      </c>
+      <c r="D16" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>Fail</v>
+      </c>
+      <c r="E16" s="3" t="str" cm="1">
+        <f t="array" ref="E16">_xlfn.IFS(ISTEXT(B16),"No  Data",B16&gt;=90,"Excellent",B16&gt;=75,"Very Good",B16&gt;50,"Good",B16&gt;40,"Average",B16&lt;40,"Fail")</f>
+        <v>Fail</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3">
+        <v>67</v>
+      </c>
+      <c r="C17" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Good</v>
+      </c>
+      <c r="D17" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>Good</v>
+      </c>
+      <c r="E17" s="3" t="str" cm="1">
+        <f t="array" ref="E17">_xlfn.IFS(ISTEXT(B17),"No  Data",B17&gt;=90,"Excellent",B17&gt;=75,"Very Good",B17&gt;50,"Good",B17&gt;40,"Average",B17&lt;40,"Fail")</f>
+        <v>Good</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J17" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3">
+        <v>79</v>
+      </c>
+      <c r="C18" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Very Good</v>
+      </c>
+      <c r="D18" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>Very Good</v>
+      </c>
+      <c r="E18" s="3" t="str" cm="1">
+        <f t="array" ref="E18">_xlfn.IFS(ISTEXT(B18),"No  Data",B18&gt;=90,"Excellent",B18&gt;=75,"Very Good",B18&gt;50,"Good",B18&gt;40,"Average",B18&lt;40,"Fail")</f>
+        <v>Very Good</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3">
+        <v>22</v>
+      </c>
+      <c r="C19" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Fail</v>
+      </c>
+      <c r="D19" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>Fail</v>
+      </c>
+      <c r="E19" s="3" t="str" cm="1">
+        <f t="array" ref="E19">_xlfn.IFS(ISTEXT(B19),"No  Data",B19&gt;=90,"Excellent",B19&gt;=75,"Very Good",B19&gt;50,"Good",B19&gt;40,"Average",B19&lt;40,"Fail")</f>
+        <v>Fail</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="3">
+        <v>90</v>
+      </c>
+      <c r="C20" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Excellent</v>
+      </c>
+      <c r="D20" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>Excellent</v>
+      </c>
+      <c r="E20" s="3" t="str" cm="1">
+        <f t="array" ref="E20">_xlfn.IFS(ISTEXT(B20),"No  Data",B20&gt;=90,"Excellent",B20&gt;=75,"Very Good",B20&gt;50,"Good",B20&gt;40,"Average",B20&lt;40,"Fail")</f>
+        <v>Excellent</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3">
+        <v>78</v>
+      </c>
+      <c r="C21" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>Very Good</v>
+      </c>
+      <c r="D21" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>Very Good</v>
+      </c>
+      <c r="E21" s="3" t="str" cm="1">
+        <f t="array" ref="E21">_xlfn.IFS(ISTEXT(B21),"No  Data",B21&gt;=90,"Excellent",B21&gt;=75,"Very Good",B21&gt;50,"Good",B21&gt;40,"Average",B21&lt;40,"Fail")</f>
+        <v>Very Good</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="3" t="str">
+        <f t="shared" si="2"/>
+        <v>No Grade</v>
+      </c>
+      <c r="D22" s="3" t="str">
+        <f t="shared" si="3"/>
+        <v>No Data</v>
+      </c>
+      <c r="E22" s="3" t="str" cm="1">
+        <f t="array" ref="E22">_xlfn.IFS(ISTEXT(B22),"No  Data",B22&gt;=90,"Excellent",B22&gt;=75,"Very Good",B22&gt;50,"Good",B22&gt;40,"Average",B22&lt;40,"Fail")</f>
+        <v>No  Data</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>